<commit_message>
BRD-13 Data Migration document set: layout fixes, register references, no account codes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.0.xlsx
+++ b/docs/deliverables/out/Migration/BIBS_Migration_BRD-13_Cutover_Task_Plan_v1.0.xlsx
@@ -7876,12 +7876,12 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>BDOI IT (legacy systems</t>
+          <t>BDOI IT (legacy systems, extracts, network, SFTP)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>extracts</t>
+          <t>BDOI</t>
         </is>
       </c>
       <c r="D13" s="12" t="n"/>
@@ -7930,12 +7930,12 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT Migration Lead (loaders</t>
+          <t>iorta TechNXT Migration Lead (loaders, reconciliation, console)</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>reconciliation</t>
+          <t>iorta TechNXT</t>
         </is>
       </c>
       <c r="D16" s="12" t="n"/>
@@ -7948,12 +7948,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT Migration Operator (intake</t>
+          <t>iorta TechNXT Migration Operator (intake, validation, loads)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>validation</t>
+          <t>iorta TechNXT</t>
         </is>
       </c>
       <c r="D17" s="12" t="n"/>
@@ -7966,12 +7966,12 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT DevOps (AWS environment</t>
+          <t>iorta TechNXT DevOps (AWS environment, snapshots, access, monitoring)</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>snapshots</t>
+          <t>iorta TechNXT</t>
         </is>
       </c>
       <c r="D18" s="12" t="n"/>
@@ -7984,12 +7984,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>iorta TechNXT QA (smoke tests</t>
+          <t>iorta TechNXT QA (smoke tests, defect triage)</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>defect triage)</t>
+          <t>iorta TechNXT</t>
         </is>
       </c>
       <c r="D19" s="12" t="n"/>

</xml_diff>